<commit_message>
refactor: semantic CSS tokens, purge dead CSS, PhaseCard/SectionHeader components
Tasks 1.1-1.3, 4.1b, 4.2b, 5.1b, 3.1b-3.3b from note1.xlsx. Zero visual
change proven: rendered HTML byte-identical before/after. globals.css
1568 -> 1072 lines; all color values now flow through --color-* tokens.

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/note1.xlsx
+++ b/note1.xlsx
@@ -1280,7 +1280,7 @@
       </c>
       <c r="H21" s="5" t="inlineStr">
         <is>
-          <t>Chưa bắt đầu</t>
+          <t>Hoàn thành</t>
         </is>
       </c>
     </row>
@@ -1424,7 +1424,7 @@
       </c>
       <c r="H25" s="5" t="inlineStr">
         <is>
-          <t>Chưa bắt đầu</t>
+          <t>Hoàn thành</t>
         </is>
       </c>
     </row>
@@ -1460,7 +1460,7 @@
       </c>
       <c r="H26" s="5" t="inlineStr">
         <is>
-          <t>Chưa bắt đầu</t>
+          <t>Hoàn thành</t>
         </is>
       </c>
     </row>
@@ -1758,7 +1758,7 @@
       </c>
       <c r="H36" s="5" t="inlineStr">
         <is>
-          <t>Chưa bắt đầu</t>
+          <t>Hoàn thành</t>
         </is>
       </c>
     </row>
@@ -1798,7 +1798,7 @@
       </c>
       <c r="H37" s="5" t="inlineStr">
         <is>
-          <t>Chưa bắt đầu</t>
+          <t>Hoàn thành</t>
         </is>
       </c>
     </row>
@@ -1838,7 +1838,7 @@
       </c>
       <c r="H38" s="5" t="inlineStr">
         <is>
-          <t>Chưa bắt đầu</t>
+          <t>Hoàn thành</t>
         </is>
       </c>
     </row>
@@ -1878,7 +1878,7 @@
       </c>
       <c r="H39" s="5" t="inlineStr">
         <is>
-          <t>Chưa bắt đầu</t>
+          <t>Hoàn thành</t>
         </is>
       </c>
     </row>
@@ -1932,7 +1932,7 @@
       </c>
       <c r="H41" s="5" t="inlineStr">
         <is>
-          <t>Chưa bắt đầu</t>
+          <t>Hoàn thành</t>
         </is>
       </c>
     </row>
@@ -2052,7 +2052,7 @@
       </c>
       <c r="H44" s="5" t="inlineStr">
         <is>
-          <t>Chưa bắt đầu</t>
+          <t>Hoàn thành</t>
         </is>
       </c>
     </row>
@@ -2106,7 +2106,7 @@
       </c>
       <c r="H46" s="5" t="inlineStr">
         <is>
-          <t>Chưa bắt đầu</t>
+          <t>Hoàn thành</t>
         </is>
       </c>
     </row>
@@ -2146,7 +2146,7 @@
       </c>
       <c r="H47" s="5" t="inlineStr">
         <is>
-          <t>Chưa bắt đầu</t>
+          <t>Hoàn thành</t>
         </is>
       </c>
     </row>
@@ -2186,7 +2186,7 @@
       </c>
       <c r="H48" s="5" t="inlineStr">
         <is>
-          <t>Chưa bắt đầu</t>
+          <t>Hoàn thành</t>
         </is>
       </c>
     </row>
@@ -2828,7 +2828,7 @@
       </c>
       <c r="H66" s="5" t="inlineStr">
         <is>
-          <t>Chưa bắt đầu</t>
+          <t>Hoàn thành</t>
         </is>
       </c>
     </row>
@@ -3172,7 +3172,7 @@
       </c>
       <c r="H76" s="5" t="inlineStr">
         <is>
-          <t>Chưa bắt đầu</t>
+          <t>Hoàn thành</t>
         </is>
       </c>
     </row>
@@ -3207,7 +3207,7 @@
       </c>
       <c r="H77" s="5" t="inlineStr">
         <is>
-          <t>Chưa bắt đầu</t>
+          <t>Hoàn thành</t>
         </is>
       </c>
     </row>
@@ -3427,6 +3427,7 @@
         </is>
       </c>
     </row>
+    <row r="84"/>
     <row r="85">
       <c r="A85" s="22" t="inlineStr">
         <is>
@@ -3454,23 +3455,23 @@
   </sheetData>
   <autoFilter ref="A1:H75"/>
   <mergeCells count="17">
+    <mergeCell ref="C13:F13"/>
+    <mergeCell ref="C40:F40"/>
+    <mergeCell ref="C9:F9"/>
+    <mergeCell ref="C45:F45"/>
     <mergeCell ref="C61:F61"/>
+    <mergeCell ref="C56:F56"/>
     <mergeCell ref="C86:G86"/>
-    <mergeCell ref="C13:F13"/>
+    <mergeCell ref="C35:F35"/>
+    <mergeCell ref="C20:F20"/>
+    <mergeCell ref="A85:B85"/>
     <mergeCell ref="C6:F6"/>
     <mergeCell ref="C30:F30"/>
     <mergeCell ref="C68:F68"/>
-    <mergeCell ref="C45:F45"/>
-    <mergeCell ref="C35:F35"/>
-    <mergeCell ref="C20:F20"/>
-    <mergeCell ref="A85:B85"/>
     <mergeCell ref="C16:F16"/>
-    <mergeCell ref="C50:F50"/>
-    <mergeCell ref="C40:F40"/>
-    <mergeCell ref="C9:F9"/>
-    <mergeCell ref="C56:F56"/>
     <mergeCell ref="C27:F27"/>
     <mergeCell ref="C2:F2"/>
+    <mergeCell ref="C50:F50"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
chore: mark completed backlog items in note1.xlsx
Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/note1.xlsx
+++ b/note1.xlsx
@@ -742,7 +742,7 @@
       </c>
       <c r="H3" s="5" t="inlineStr">
         <is>
-          <t>Chưa bắt đầu</t>
+          <t>Hoàn thành</t>
         </is>
       </c>
     </row>
@@ -778,7 +778,7 @@
       </c>
       <c r="H4" s="5" t="inlineStr">
         <is>
-          <t>Chưa bắt đầu</t>
+          <t>Hoàn thành</t>
         </is>
       </c>
     </row>
@@ -814,7 +814,7 @@
       </c>
       <c r="H5" s="5" t="inlineStr">
         <is>
-          <t>Chưa bắt đầu</t>
+          <t>Hoàn thành</t>
         </is>
       </c>
     </row>
@@ -950,7 +950,7 @@
       </c>
       <c r="H10" s="5" t="inlineStr">
         <is>
-          <t>Chưa bắt đầu</t>
+          <t>Hoàn thành</t>
         </is>
       </c>
     </row>
@@ -986,7 +986,7 @@
       </c>
       <c r="H11" s="5" t="inlineStr">
         <is>
-          <t>Chưa bắt đầu</t>
+          <t>Hoàn thành</t>
         </is>
       </c>
     </row>
@@ -1022,7 +1022,7 @@
       </c>
       <c r="H12" s="5" t="inlineStr">
         <is>
-          <t>Chưa bắt đầu</t>
+          <t>Hoàn thành</t>
         </is>
       </c>
     </row>
@@ -1158,7 +1158,7 @@
       </c>
       <c r="H17" s="5" t="inlineStr">
         <is>
-          <t>Chưa bắt đầu</t>
+          <t>Hoàn thành</t>
         </is>
       </c>
     </row>
@@ -1194,7 +1194,7 @@
       </c>
       <c r="H18" s="5" t="inlineStr">
         <is>
-          <t>Chưa bắt đầu</t>
+          <t>Hoàn thành</t>
         </is>
       </c>
     </row>
@@ -1230,7 +1230,7 @@
       </c>
       <c r="H19" s="5" t="inlineStr">
         <is>
-          <t>Chưa bắt đầu</t>
+          <t>Hoàn thành</t>
         </is>
       </c>
     </row>
@@ -1316,7 +1316,7 @@
       </c>
       <c r="H22" s="5" t="inlineStr">
         <is>
-          <t>Chưa bắt đầu</t>
+          <t>Hoàn thành</t>
         </is>
       </c>
     </row>
@@ -1352,7 +1352,7 @@
       </c>
       <c r="H23" s="5" t="inlineStr">
         <is>
-          <t>Chưa bắt đầu</t>
+          <t>Hoàn thành</t>
         </is>
       </c>
     </row>
@@ -1972,7 +1972,7 @@
       </c>
       <c r="H42" s="5" t="inlineStr">
         <is>
-          <t>Chưa bắt đầu</t>
+          <t>Hoàn thành</t>
         </is>
       </c>
     </row>
@@ -2012,7 +2012,7 @@
       </c>
       <c r="H43" s="5" t="inlineStr">
         <is>
-          <t>Chưa bắt đầu</t>
+          <t>Hoàn thành</t>
         </is>
       </c>
     </row>
@@ -2280,7 +2280,7 @@
       </c>
       <c r="H51" s="5" t="inlineStr">
         <is>
-          <t>Chưa bắt đầu</t>
+          <t>Hoàn thành</t>
         </is>
       </c>
     </row>
@@ -2320,7 +2320,7 @@
       </c>
       <c r="H52" s="5" t="inlineStr">
         <is>
-          <t>Chưa bắt đầu</t>
+          <t>Hoàn thành</t>
         </is>
       </c>
     </row>
@@ -2360,7 +2360,7 @@
       </c>
       <c r="H53" s="5" t="inlineStr">
         <is>
-          <t>Chưa bắt đầu</t>
+          <t>Hoàn thành</t>
         </is>
       </c>
     </row>
@@ -2494,7 +2494,7 @@
       </c>
       <c r="H57" s="5" t="inlineStr">
         <is>
-          <t>Chưa bắt đầu</t>
+          <t>Hoàn thành</t>
         </is>
       </c>
     </row>
@@ -2534,7 +2534,7 @@
       </c>
       <c r="H58" s="5" t="inlineStr">
         <is>
-          <t>Chưa bắt đầu</t>
+          <t>Hoàn thành</t>
         </is>
       </c>
     </row>
@@ -2574,7 +2574,7 @@
       </c>
       <c r="H59" s="5" t="inlineStr">
         <is>
-          <t>Chưa bắt đầu</t>
+          <t>Hoàn thành</t>
         </is>
       </c>
     </row>
@@ -2668,7 +2668,7 @@
       </c>
       <c r="H62" s="5" t="inlineStr">
         <is>
-          <t>Chưa bắt đầu</t>
+          <t>Hoàn thành</t>
         </is>
       </c>
     </row>
@@ -2748,7 +2748,7 @@
       </c>
       <c r="H64" s="5" t="inlineStr">
         <is>
-          <t>Chưa bắt đầu</t>
+          <t>Hoàn thành</t>
         </is>
       </c>
     </row>
@@ -2788,7 +2788,7 @@
       </c>
       <c r="H65" s="5" t="inlineStr">
         <is>
-          <t>Chưa bắt đầu</t>
+          <t>Hoàn thành</t>
         </is>
       </c>
     </row>
@@ -2922,7 +2922,7 @@
       </c>
       <c r="H69" s="5" t="inlineStr">
         <is>
-          <t>Chưa bắt đầu</t>
+          <t>Hoàn thành</t>
         </is>
       </c>
     </row>
@@ -3042,7 +3042,7 @@
       </c>
       <c r="H72" s="5" t="inlineStr">
         <is>
-          <t>Chưa bắt đầu</t>
+          <t>Hoàn thành</t>
         </is>
       </c>
     </row>
@@ -3122,7 +3122,7 @@
       </c>
       <c r="H74" s="5" t="inlineStr">
         <is>
-          <t>Chưa bắt đầu</t>
+          <t>Hoàn thành</t>
         </is>
       </c>
     </row>
@@ -3243,7 +3243,7 @@
       </c>
       <c r="H78" s="5" t="inlineStr">
         <is>
-          <t>Chưa bắt đầu</t>
+          <t>Hoàn thành</t>
         </is>
       </c>
     </row>
@@ -3279,7 +3279,7 @@
       </c>
       <c r="H79" s="5" t="inlineStr">
         <is>
-          <t>Chưa bắt đầu</t>
+          <t>Hoàn thành</t>
         </is>
       </c>
     </row>

</xml_diff>